<commit_message>
fix(advi): perfeccionamiento metodologico convergencia elbo moran comparacion advi nuts y consistencia
</commit_message>
<xml_diff>
--- a/outputs/tables/tabla_comparacion_advi_nuts.xlsx
+++ b/outputs/tables/tabla_comparacion_advi_nuts.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
+  <si>
+    <t>Modelo</t>
+  </si>
   <si>
     <t>Parámetro</t>
   </si>
@@ -37,12 +40,24 @@
     <t>HDI_95_NUTS</t>
   </si>
   <si>
+    <t>Diferencia_Relativa_Medias_Pct</t>
+  </si>
+  <si>
     <t>Ratio_SD (ADVI/NUTS)</t>
   </si>
   <si>
     <t>Subestimacion_Incertidumbre_Pct</t>
   </si>
   <si>
+    <t>HDI_ADVI_Contiene_Media_NUTS</t>
+  </si>
+  <si>
+    <t>Modelo (c) Besag ICAR + No Estructurado (Mejor LOO)</t>
+  </si>
+  <si>
+    <t>Modelo (d) BYM2 (Prior Beta(0.5, 0.5))</t>
+  </si>
+  <si>
     <t>Intercepto Cantonal (alpha)</t>
   </si>
   <si>
@@ -52,67 +67,130 @@
     <t>Elasticidad Área Territorial (beta_area)</t>
   </si>
   <si>
-    <t>Escala Espacial BYM2 (sigma_s)</t>
-  </si>
-  <si>
-    <t>Parámetro de Mezcla Espacial (rho)</t>
+    <t>Escala Espacial ICAR (sigma_phi)</t>
+  </si>
+  <si>
+    <t>Escala Efecto No Estructurado (sigma_theta)</t>
   </si>
   <si>
     <t>Dispersión Binomial Negativa (alpha_disp)</t>
   </si>
   <si>
-    <t>[1.5327, 1.7101]</t>
-  </si>
-  <si>
-    <t>[0.1995, 0.4422]</t>
-  </si>
-  <si>
-    <t>[0.0510, 0.1734]</t>
-  </si>
-  <si>
-    <t>[0.8449, 1.0320]</t>
-  </si>
-  <si>
-    <t>[0.0009, 0.1485]</t>
-  </si>
-  <si>
-    <t>[1.5588, 2.3266]</t>
-  </si>
-  <si>
-    <t>[1.2374, 1.4995]</t>
-  </si>
-  <si>
-    <t>[0.1903, 0.4278]</t>
-  </si>
-  <si>
-    <t>[0.0939, 0.3820]</t>
-  </si>
-  <si>
-    <t>[1.2423, 1.8463]</t>
-  </si>
-  <si>
-    <t>[0.5891, 0.9892]</t>
-  </si>
-  <si>
-    <t>[3.8136, 7.3525]</t>
-  </si>
-  <si>
-    <t>+32.6%</t>
-  </si>
-  <si>
-    <t>-1.7%</t>
-  </si>
-  <si>
-    <t>+57.8%</t>
-  </si>
-  <si>
-    <t>+69.7%</t>
-  </si>
-  <si>
-    <t>+59.2%</t>
-  </si>
-  <si>
-    <t>+79.0%</t>
+    <t>Escala Espacial Total BYM2 (sigma_s)</t>
+  </si>
+  <si>
+    <t>Parámetro de Mezcla Espacial Beta(0.5, 0.5) (rho)</t>
+  </si>
+  <si>
+    <t>[1.2811, 1.3805]</t>
+  </si>
+  <si>
+    <t>[0.2438, 0.3853]</t>
+  </si>
+  <si>
+    <t>[0.2788, 0.3617]</t>
+  </si>
+  <si>
+    <t>[2.4639, 2.6605]</t>
+  </si>
+  <si>
+    <t>[0.0036, 0.0607]</t>
+  </si>
+  <si>
+    <t>[5.5396, 9.1767]</t>
+  </si>
+  <si>
+    <t>[1.2817, 1.3812]</t>
+  </si>
+  <si>
+    <t>[0.2436, 0.3856]</t>
+  </si>
+  <si>
+    <t>[0.2788, 0.3613]</t>
+  </si>
+  <si>
+    <t>[2.1384, 2.3089]</t>
+  </si>
+  <si>
+    <t>[0.9991, 1.0000]</t>
+  </si>
+  <si>
+    <t>[5.5562, 9.1987]</t>
+  </si>
+  <si>
+    <t>[1.2433, 1.4991]</t>
+  </si>
+  <si>
+    <t>[0.1934, 0.4225]</t>
+  </si>
+  <si>
+    <t>[0.0959, 0.3861]</t>
+  </si>
+  <si>
+    <t>[1.1373, 2.0912]</t>
+  </si>
+  <si>
+    <t>[0.1196, 0.8542]</t>
+  </si>
+  <si>
+    <t>[3.7865, 7.2327]</t>
+  </si>
+  <si>
+    <t>[1.2449, 1.4973]</t>
+  </si>
+  <si>
+    <t>[0.1926, 0.4336]</t>
+  </si>
+  <si>
+    <t>[0.0918, 0.3782]</t>
+  </si>
+  <si>
+    <t>[1.2232, 1.8205]</t>
+  </si>
+  <si>
+    <t>[0.5762, 0.9932]</t>
+  </si>
+  <si>
+    <t>[3.8222, 7.2670]</t>
+  </si>
+  <si>
+    <t>+61.4%</t>
+  </si>
+  <si>
+    <t>+38.0%</t>
+  </si>
+  <si>
+    <t>+70.9%</t>
+  </si>
+  <si>
+    <t>+79.8%</t>
+  </si>
+  <si>
+    <t>+90.8%</t>
+  </si>
+  <si>
+    <t>-3.4%</t>
+  </si>
+  <si>
+    <t>+61.3%</t>
+  </si>
+  <si>
+    <t>+41.1%</t>
+  </si>
+  <si>
+    <t>+72.5%</t>
+  </si>
+  <si>
+    <t>+99.3%</t>
+  </si>
+  <si>
+    <t>-0.8%</t>
+  </si>
+  <si>
+    <t>SÍ</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -470,10 +548,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,179 +579,470 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2">
-        <v>1.6235</v>
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
       </c>
       <c r="C2">
-        <v>0.0449</v>
-      </c>
-      <c r="D2" t="s">
+        <v>1.332</v>
+      </c>
+      <c r="D2">
+        <v>0.0252</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2">
+        <v>1.3703</v>
+      </c>
+      <c r="G2">
+        <v>0.06510000000000001</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>-2.79</v>
+      </c>
+      <c r="J2">
+        <v>0.3863</v>
+      </c>
+      <c r="K2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>15</v>
       </c>
-      <c r="E2">
-        <v>1.3701</v>
-      </c>
-      <c r="F2">
-        <v>0.0667</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2">
-        <v>0.6737</v>
-      </c>
-      <c r="I2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
-        <v>0.3175</v>
-      </c>
       <c r="C3">
-        <v>0.0613</v>
-      </c>
-      <c r="D3" t="s">
+        <v>0.3126</v>
+      </c>
+      <c r="D3">
+        <v>0.0357</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3">
+        <v>0.3101</v>
+      </c>
+      <c r="G3">
+        <v>0.0577</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3">
+        <v>0.79</v>
+      </c>
+      <c r="J3">
+        <v>0.62</v>
+      </c>
+      <c r="K3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="E3">
-        <v>0.3093</v>
-      </c>
-      <c r="F3">
-        <v>0.0603</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3">
-        <v>1.0172</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4">
-        <v>0.114</v>
-      </c>
       <c r="C4">
-        <v>0.0316</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4">
-        <v>0.2306</v>
+        <v>0.3215</v>
+      </c>
+      <c r="D4">
+        <v>0.0214</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
       </c>
       <c r="F4">
-        <v>0.075</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4">
-        <v>0.422</v>
-      </c>
-      <c r="I4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>0.2322</v>
+      </c>
+      <c r="G4">
+        <v>0.0737</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4">
+        <v>38.45</v>
+      </c>
+      <c r="J4">
+        <v>0.2906</v>
+      </c>
+      <c r="K4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5">
-        <v>0.9327</v>
+      <c r="B5" t="s">
+        <v>17</v>
       </c>
       <c r="C5">
-        <v>0.047</v>
-      </c>
-      <c r="D5" t="s">
+        <v>2.5583</v>
+      </c>
+      <c r="D5">
+        <v>0.0494</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>1.5868</v>
+      </c>
+      <c r="G5">
+        <v>0.244</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5">
+        <v>61.22</v>
+      </c>
+      <c r="J5">
+        <v>0.2025</v>
+      </c>
+      <c r="K5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="E5">
-        <v>1.4986</v>
-      </c>
-      <c r="F5">
-        <v>0.1553</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5">
-        <v>0.3025</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="C6">
+        <v>0.0192</v>
+      </c>
+      <c r="D6">
+        <v>0.0155</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6">
+        <v>0.5803</v>
+      </c>
+      <c r="G6">
+        <v>0.1688</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6">
+        <v>-96.69</v>
+      </c>
+      <c r="J6">
+        <v>0.0917</v>
+      </c>
+      <c r="K6" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7">
+        <v>7.0989</v>
+      </c>
+      <c r="D7">
+        <v>0.8997000000000001</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7">
+        <v>5.3233</v>
+      </c>
+      <c r="G7">
+        <v>0.8704</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7">
+        <v>33.35</v>
+      </c>
+      <c r="J7">
+        <v>1.0337</v>
+      </c>
+      <c r="K7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8">
+        <v>1.3327</v>
+      </c>
+      <c r="D8">
+        <v>0.0252</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8">
+        <v>1.3702</v>
+      </c>
+      <c r="G8">
+        <v>0.065</v>
+      </c>
+      <c r="H8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8">
+        <v>-2.74</v>
+      </c>
+      <c r="J8">
+        <v>0.387</v>
+      </c>
+      <c r="K8" t="s">
+        <v>52</v>
+      </c>
+      <c r="L8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>0.3126</v>
+      </c>
+      <c r="D9">
+        <v>0.0359</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9">
+        <v>0.3112</v>
+      </c>
+      <c r="G9">
+        <v>0.0609</v>
+      </c>
+      <c r="H9" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9">
+        <v>0.45</v>
+      </c>
+      <c r="J9">
+        <v>0.5891999999999999</v>
+      </c>
+      <c r="K9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>0.3212</v>
+      </c>
+      <c r="D10">
+        <v>0.0213</v>
+      </c>
+      <c r="E10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
+      <c r="F10">
+        <v>0.2299</v>
+      </c>
+      <c r="G10">
+        <v>0.0733</v>
+      </c>
+      <c r="H10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10">
+        <v>39.73</v>
+      </c>
+      <c r="J10">
+        <v>0.2908</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B6">
-        <v>0.0274</v>
-      </c>
-      <c r="C6">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>2.2203</v>
+      </c>
+      <c r="D11">
         <v>0.0429</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11">
+        <v>1.4992</v>
+      </c>
+      <c r="G11">
+        <v>0.1559</v>
+      </c>
+      <c r="H11" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11">
+        <v>48.1</v>
+      </c>
+      <c r="J11">
+        <v>0.2749</v>
+      </c>
+      <c r="K11" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12">
+        <v>0.9998</v>
+      </c>
+      <c r="D12">
+        <v>0.0007</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12">
+        <v>0.8199</v>
+      </c>
+      <c r="G12">
+        <v>0.1055</v>
+      </c>
+      <c r="H12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I12">
+        <v>21.94</v>
+      </c>
+      <c r="J12">
+        <v>0.0069</v>
+      </c>
+      <c r="K12" t="s">
+        <v>55</v>
+      </c>
+      <c r="L12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
         <v>19</v>
       </c>
-      <c r="E6">
-        <v>0.8127</v>
-      </c>
-      <c r="F6">
-        <v>0.1052</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6">
-        <v>0.4078</v>
-      </c>
-      <c r="I6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7">
-        <v>1.8953</v>
-      </c>
-      <c r="C7">
-        <v>0.1903</v>
-      </c>
-      <c r="D7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7">
-        <v>5.3588</v>
-      </c>
-      <c r="F7">
-        <v>0.9064</v>
-      </c>
-      <c r="G7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7">
-        <v>0.2099</v>
-      </c>
-      <c r="I7" t="s">
-        <v>32</v>
+      <c r="C13">
+        <v>7.118</v>
+      </c>
+      <c r="D13">
+        <v>0.9011</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13">
+        <v>5.3177</v>
+      </c>
+      <c r="G13">
+        <v>0.8944</v>
+      </c>
+      <c r="H13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13">
+        <v>33.85</v>
+      </c>
+      <c r="J13">
+        <v>1.0075</v>
+      </c>
+      <c r="K13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L13" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(pipeline): consolidar modelo b como ganador loo, validacion nuts y calibracion de incertidumbre
</commit_message>
<xml_diff>
--- a/outputs/tables/tabla_comparacion_advi_nuts.xlsx
+++ b/outputs/tables/tabla_comparacion_advi_nuts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
   <si>
     <t>Modelo</t>
   </si>
@@ -52,7 +52,10 @@
     <t>HDI_ADVI_Contiene_Media_NUTS</t>
   </si>
   <si>
-    <t>Modelo (c) Besag ICAR + No Estructurado (Mejor LOO)</t>
+    <t>Modelo (b) Binomial Negativa (ICAR) [Mejor LOO]</t>
+  </si>
+  <si>
+    <t>Modelo (c) Besag ICAR + No Estructurado</t>
   </si>
   <si>
     <t>Modelo (d) BYM2 (Prior Beta(0.5, 0.5))</t>
@@ -70,18 +73,33 @@
     <t>Escala Espacial ICAR (sigma_phi)</t>
   </si>
   <si>
+    <t>Dispersión Binomial Negativa (alpha_disp)</t>
+  </si>
+  <si>
     <t>Escala Efecto No Estructurado (sigma_theta)</t>
   </si>
   <si>
-    <t>Dispersión Binomial Negativa (alpha_disp)</t>
-  </si>
-  <si>
     <t>Escala Espacial Total BYM2 (sigma_s)</t>
   </si>
   <si>
     <t>Parámetro de Mezcla Espacial Beta(0.5, 0.5) (rho)</t>
   </si>
   <si>
+    <t>[1.2997, 1.3982]</t>
+  </si>
+  <si>
+    <t>[0.2521, 0.3922]</t>
+  </si>
+  <si>
+    <t>[0.2865, 0.3623]</t>
+  </si>
+  <si>
+    <t>[2.4965, 2.7038]</t>
+  </si>
+  <si>
+    <t>[5.4081, 8.7699]</t>
+  </si>
+  <si>
     <t>[1.2811, 1.3805]</t>
   </si>
   <si>
@@ -118,6 +136,21 @@
     <t>[5.5562, 9.1987]</t>
   </si>
   <si>
+    <t>[1.2696, 1.4681]</t>
+  </si>
+  <si>
+    <t>[0.1982, 0.4211]</t>
+  </si>
+  <si>
+    <t>[0.2034, 0.4555]</t>
+  </si>
+  <si>
+    <t>[1.8026, 2.3235]</t>
+  </si>
+  <si>
+    <t>[3.6346, 7.0755]</t>
+  </si>
+  <si>
     <t>[1.2433, 1.4991]</t>
   </si>
   <si>
@@ -152,6 +185,21 @@
   </si>
   <si>
     <t>[3.8222, 7.2670]</t>
+  </si>
+  <si>
+    <t>+50.9%</t>
+  </si>
+  <si>
+    <t>+38.2%</t>
+  </si>
+  <si>
+    <t>+69.5%</t>
+  </si>
+  <si>
+    <t>+61.0%</t>
+  </si>
+  <si>
+    <t>-1.0%</t>
   </si>
   <si>
     <t>+61.4%</t>
@@ -548,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -594,37 +642,37 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2">
-        <v>1.332</v>
+        <v>1.3482</v>
       </c>
       <c r="D2">
-        <v>0.0252</v>
+        <v>0.0249</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2">
-        <v>1.3703</v>
+        <v>1.3682</v>
       </c>
       <c r="G2">
-        <v>0.06510000000000001</v>
+        <v>0.0507</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="I2">
-        <v>-2.79</v>
+        <v>-1.46</v>
       </c>
       <c r="J2">
-        <v>0.3863</v>
+        <v>0.4907</v>
       </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="L2" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -632,37 +680,37 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3">
-        <v>0.3126</v>
+        <v>0.3207</v>
       </c>
       <c r="D3">
-        <v>0.0357</v>
+        <v>0.036</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3">
-        <v>0.3101</v>
+        <v>0.3104</v>
       </c>
       <c r="G3">
-        <v>0.0577</v>
+        <v>0.0582</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="I3">
-        <v>0.79</v>
+        <v>3.34</v>
       </c>
       <c r="J3">
-        <v>0.62</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="K3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="L3" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -670,37 +718,37 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
-        <v>0.3215</v>
+        <v>0.3242</v>
       </c>
       <c r="D4">
-        <v>0.0214</v>
+        <v>0.0196</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4">
-        <v>0.2322</v>
+        <v>0.3223</v>
       </c>
       <c r="G4">
-        <v>0.0737</v>
+        <v>0.0641</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="I4">
-        <v>38.45</v>
+        <v>0.6</v>
       </c>
       <c r="J4">
-        <v>0.2906</v>
+        <v>0.305</v>
       </c>
       <c r="K4" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="L4" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -708,37 +756,37 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5">
-        <v>2.5583</v>
+        <v>2.5948</v>
       </c>
       <c r="D5">
-        <v>0.0494</v>
+        <v>0.0523</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5">
-        <v>1.5868</v>
+        <v>2.0494</v>
       </c>
       <c r="G5">
-        <v>0.244</v>
+        <v>0.1342</v>
       </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="I5">
-        <v>61.22</v>
+        <v>26.61</v>
       </c>
       <c r="J5">
-        <v>0.2025</v>
+        <v>0.3896</v>
       </c>
       <c r="K5" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="L5" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -746,75 +794,75 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>0.0192</v>
+        <v>6.9813</v>
       </c>
       <c r="D6">
-        <v>0.0155</v>
+        <v>0.8838</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6">
-        <v>0.5803</v>
+        <v>5.1165</v>
       </c>
       <c r="G6">
-        <v>0.1688</v>
+        <v>0.8751</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="I6">
-        <v>-96.69</v>
+        <v>36.45</v>
       </c>
       <c r="J6">
-        <v>0.0917</v>
+        <v>1.01</v>
       </c>
       <c r="K6" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="L6" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C7">
-        <v>7.0989</v>
+        <v>1.332</v>
       </c>
       <c r="D7">
-        <v>0.8997000000000001</v>
+        <v>0.0252</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F7">
-        <v>5.3233</v>
+        <v>1.3703</v>
       </c>
       <c r="G7">
-        <v>0.8704</v>
+        <v>0.06510000000000001</v>
       </c>
       <c r="H7" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I7">
-        <v>33.35</v>
+        <v>-2.79</v>
       </c>
       <c r="J7">
-        <v>1.0337</v>
+        <v>0.3863</v>
       </c>
       <c r="K7" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="L7" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -822,37 +870,37 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8">
-        <v>1.3327</v>
+        <v>0.3126</v>
       </c>
       <c r="D8">
-        <v>0.0252</v>
+        <v>0.0357</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8">
-        <v>1.3702</v>
+        <v>0.3101</v>
       </c>
       <c r="G8">
-        <v>0.065</v>
+        <v>0.0577</v>
       </c>
       <c r="H8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="I8">
-        <v>-2.74</v>
+        <v>0.79</v>
       </c>
       <c r="J8">
-        <v>0.387</v>
+        <v>0.62</v>
       </c>
       <c r="K8" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="L8" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -860,37 +908,37 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9">
-        <v>0.3126</v>
+        <v>0.3215</v>
       </c>
       <c r="D9">
-        <v>0.0359</v>
+        <v>0.0214</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9">
-        <v>0.3112</v>
+        <v>0.2322</v>
       </c>
       <c r="G9">
-        <v>0.0609</v>
+        <v>0.0737</v>
       </c>
       <c r="H9" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I9">
-        <v>0.45</v>
+        <v>38.45</v>
       </c>
       <c r="J9">
-        <v>0.5891999999999999</v>
+        <v>0.2906</v>
       </c>
       <c r="K9" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="L9" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -898,37 +946,37 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C10">
-        <v>0.3212</v>
+        <v>2.5583</v>
       </c>
       <c r="D10">
-        <v>0.0213</v>
+        <v>0.0494</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F10">
-        <v>0.2299</v>
+        <v>1.5868</v>
       </c>
       <c r="G10">
-        <v>0.0733</v>
+        <v>0.244</v>
       </c>
       <c r="H10" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I10">
-        <v>39.73</v>
+        <v>61.22</v>
       </c>
       <c r="J10">
-        <v>0.2908</v>
+        <v>0.2025</v>
       </c>
       <c r="K10" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="L10" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -939,34 +987,34 @@
         <v>20</v>
       </c>
       <c r="C11">
-        <v>2.2203</v>
+        <v>0.0192</v>
       </c>
       <c r="D11">
-        <v>0.0429</v>
+        <v>0.0155</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F11">
-        <v>1.4992</v>
+        <v>0.5803</v>
       </c>
       <c r="G11">
-        <v>0.1559</v>
+        <v>0.1688</v>
       </c>
       <c r="H11" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I11">
-        <v>48.1</v>
+        <v>-96.69</v>
       </c>
       <c r="J11">
-        <v>0.2749</v>
+        <v>0.0917</v>
       </c>
       <c r="K11" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -974,75 +1022,265 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12">
-        <v>0.9998</v>
+        <v>7.0989</v>
       </c>
       <c r="D12">
-        <v>0.0007</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F12">
-        <v>0.8199</v>
+        <v>5.3233</v>
       </c>
       <c r="G12">
-        <v>0.1055</v>
+        <v>0.8704</v>
       </c>
       <c r="H12" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I12">
-        <v>21.94</v>
+        <v>33.35</v>
       </c>
       <c r="J12">
-        <v>0.0069</v>
+        <v>1.0337</v>
       </c>
       <c r="K12" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="L12" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13">
+        <v>1.3327</v>
+      </c>
+      <c r="D13">
+        <v>0.0252</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13">
+        <v>1.3702</v>
+      </c>
+      <c r="G13">
+        <v>0.065</v>
+      </c>
+      <c r="H13" t="s">
+        <v>51</v>
+      </c>
+      <c r="I13">
+        <v>-2.74</v>
+      </c>
+      <c r="J13">
+        <v>0.387</v>
+      </c>
+      <c r="K13" t="s">
+        <v>68</v>
+      </c>
+      <c r="L13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14">
+        <v>0.3126</v>
+      </c>
+      <c r="D14">
+        <v>0.0359</v>
+      </c>
+      <c r="E14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14">
+        <v>0.3112</v>
+      </c>
+      <c r="G14">
+        <v>0.0609</v>
+      </c>
+      <c r="H14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14">
+        <v>0.45</v>
+      </c>
+      <c r="J14">
+        <v>0.5891999999999999</v>
+      </c>
+      <c r="K14" t="s">
+        <v>69</v>
+      </c>
+      <c r="L14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>0.3212</v>
+      </c>
+      <c r="D15">
+        <v>0.0213</v>
+      </c>
+      <c r="E15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15">
+        <v>0.2299</v>
+      </c>
+      <c r="G15">
+        <v>0.0733</v>
+      </c>
+      <c r="H15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I15">
+        <v>39.73</v>
+      </c>
+      <c r="J15">
+        <v>0.2908</v>
+      </c>
+      <c r="K15" t="s">
+        <v>64</v>
+      </c>
+      <c r="L15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16">
+        <v>2.2203</v>
+      </c>
+      <c r="D16">
+        <v>0.0429</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16">
+        <v>1.4992</v>
+      </c>
+      <c r="G16">
+        <v>0.1559</v>
+      </c>
+      <c r="H16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I16">
+        <v>48.1</v>
+      </c>
+      <c r="J16">
+        <v>0.2749</v>
+      </c>
+      <c r="K16" t="s">
+        <v>70</v>
+      </c>
+      <c r="L16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17">
+        <v>0.9998</v>
+      </c>
+      <c r="D17">
+        <v>0.0007</v>
+      </c>
+      <c r="E17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17">
+        <v>0.8199</v>
+      </c>
+      <c r="G17">
+        <v>0.1055</v>
+      </c>
+      <c r="H17" t="s">
+        <v>55</v>
+      </c>
+      <c r="I17">
+        <v>21.94</v>
+      </c>
+      <c r="J17">
+        <v>0.0069</v>
+      </c>
+      <c r="K17" t="s">
+        <v>71</v>
+      </c>
+      <c r="L17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C13">
+      <c r="C18">
         <v>7.118</v>
       </c>
-      <c r="D13">
+      <c r="D18">
         <v>0.9011</v>
       </c>
-      <c r="E13" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13">
+      <c r="E18" t="s">
+        <v>39</v>
+      </c>
+      <c r="F18">
         <v>5.3177</v>
       </c>
-      <c r="G13">
+      <c r="G18">
         <v>0.8944</v>
       </c>
-      <c r="H13" t="s">
-        <v>45</v>
-      </c>
-      <c r="I13">
+      <c r="H18" t="s">
+        <v>56</v>
+      </c>
+      <c r="I18">
         <v>33.85</v>
       </c>
-      <c r="J13">
+      <c r="J18">
         <v>1.0075</v>
       </c>
-      <c r="K13" t="s">
-        <v>56</v>
-      </c>
-      <c r="L13" t="s">
-        <v>58</v>
+      <c r="K18" t="s">
+        <v>72</v>
+      </c>
+      <c r="L18" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>